<commit_message>
Títulos: usar la marca completa «| Aluminios Olmedo» en todas las tandas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Le6dThhENh6Yrnr8uFDqix
</commit_message>
<xml_diff>
--- a/entregables/Titulos-metas-2026-10-29.xlsx
+++ b/entregables/Titulos-metas-2026-10-29.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Título NUEVO</t>
+          <t>Título NUEVO (completo, con « | Aluminios Olmedo»)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Ventanas VELUX Giratorias | Medidas y Precios | Olmedo</t>
+          <t>VELUX Giratorias: Medidas y Precios | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L2" s="2" t="n">
@@ -675,7 +675,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Ventanas VELUX: Catálogo, Medidas y Precios | Olmedo</t>
+          <t>Ventanas VELUX: Medidas y Precios | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L3" s="2" t="n">
@@ -748,11 +748,11 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Ventana VELUX GGL 3070 Madera: Medidas y Precio | Olmedo</t>
+          <t>VELUX GGL 3070 Madera: Medidas y Precio | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
@@ -821,11 +821,11 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Persiana Eléctrica VELUX SML | Precio y Medidas | Olmedo</t>
+          <t>Persiana VELUX SML: Precio y Medidas | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L5" s="2" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
@@ -894,11 +894,11 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Escalera Recta Madera Maydisa Lisbon | Precio y Medidas</t>
+          <t>Escalera Madera Maydisa Lisbon: Precio | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
@@ -967,11 +967,11 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Ventana de Tejado Lucera Roto UNV | Olmedo</t>
+          <t>Ventana de Tejado Lucera Roto UNV | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
@@ -1040,11 +1040,11 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Estor Eléctrico VELUX RML para Tejado | Olmedo</t>
+          <t>Estor Eléctrico VELUX RML para Tejado | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L8" s="2" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
@@ -1113,11 +1113,11 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Tubo Solar VELUX 35 cm Flexible | Olmedo</t>
+          <t>Tubo Solar VELUX 35 cm Flexible | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L9" s="2" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
@@ -1186,11 +1186,11 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Ventana de Tejado Roto R45 Pivotante | Olmedo</t>
+          <t>Ventana de Tejado Roto R45 Pivotante | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L10" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
@@ -1259,11 +1259,11 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Persiana Solar VELUX SSL sin Obra | Olmedo</t>
+          <t>Persiana Solar VELUX SSL sin Obra | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L11" s="2" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
@@ -1332,11 +1332,11 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Ventana Tejado Roto R48S Vidrio Seguridad | Olmedo</t>
+          <t>Ventana Roto R48S Vidrio Seguridad | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L12" s="2" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Revisión de la estrategia SEO frente a posiciones actuales y ajuste de títulos (keyword primero, marca al final)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Le6dThhENh6Yrnr8uFDqix
</commit_message>
<xml_diff>
--- a/entregables/Titulos-metas-2026-10-29.xlsx
+++ b/entregables/Titulos-metas-2026-10-29.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Título NUEVO (completo, con « | Aluminios Olmedo»)</t>
+          <t>Título NUEVO (keyword primero, marca al final)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -602,11 +602,11 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>VELUX Giratorias: Medidas y Precios | Aluminios Olmedo</t>
+          <t>Ventanas VELUX Giratorias: Medidas y Precios | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L2" s="2" t="n">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
@@ -675,11 +675,11 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Ventanas VELUX: Medidas y Precios | Aluminios Olmedo</t>
+          <t>Ventanas VELUX de Tejado: Modelos y Precios | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L3" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
@@ -821,11 +821,11 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Persiana VELUX SML: Precio y Medidas | Aluminios Olmedo</t>
+          <t>Persiana Eléctrica VELUX SML: Precio y Medidas | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L5" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
@@ -845,7 +845,7 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Aparece por «persianas velux» (479 impresiones, 0 clics): se pone en plural y al inicio.</t>
+          <t>«persianas velux» (plural) es de la categoría 522 según la estrategia: la ficha va en singular y con el modelo.</t>
         </is>
       </c>
       <c r="R5" s="2" t="n"/>
@@ -894,11 +894,11 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Escalera Madera Maydisa Lisbon: Precio | Aluminios Olmedo</t>
+          <t>Escalera Recta de Madera Maydisa Lisbon: Precio | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
@@ -918,7 +918,7 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Título cortado («Lisb»). La búsqueda que trae clics es «escalera de madera interior».</t>
+          <t>«escalera de madera interior» es de la categoría 560 según la estrategia: la ficha va con el modelo.</t>
         </is>
       </c>
       <c r="R6" s="2" t="n"/>
@@ -967,11 +967,11 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Ventana de Tejado Lucera Roto UNV | Aluminios Olmedo</t>
+          <t>Lucera para Tejado Roto UNV Universal | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
@@ -991,7 +991,7 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>Sale por «ventanas de tejado» (678 impresiones, 1 clic). Ojo: esa búsqueda debe ganarla la categoría 503 (tarea 3.2).</t>
+          <t>Se evita «ventanas de tejado» (es de la 503) y se apunta a «luceras para tejados» (pos. 9).</t>
         </is>
       </c>
       <c r="R7" s="2" t="n"/>
@@ -1073,55 +1073,55 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>3 · opcional, desde 10-dic</t>
+          <t>2 · desde 19-nov</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://aluminio-carpinteria.com/tubo-solar-velux-cubierta-inclinada/300-tubo-solar-velux-o-35cm-flexible-cubierta-inclinada.html</t>
+          <t>https://aluminio-carpinteria.com/560-escaleras-rectas-madera</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Producto</t>
+          <t>Categoría</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1805</v>
+        <v>491</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.3</v>
+        <v>3.9</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>8</v>
+        <v>17.6</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>tubo solar velux; tubo solar; tubo solar velux precio</t>
+          <t>escalera de madera interior / escalera interior de madera (770/mes)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Tubo Solar Flexible VELUX 35cm Cubierta I | Aluminios Olmedo</t>
+          <t>Escaleras Rectas de Madera para Interior y Altillos</t>
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Tubo Solar VELUX 35 cm Flexible | Aluminios Olmedo</t>
+          <t>Escaleras de Madera Interior y para Altillos | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L9" s="2" t="n">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Tubo solar flexible VELUX Ø 35cm para cubierta inclinada. Rodea obstáculos fácilmente. Lleva luz natural al interior. Distribuidor oficial VELUX.</t>
+          <t>Comprar escalera recta de madera para interior o altillo. Modelos Maydisa resistentes, envío rápido y fácil montaje al mejor precio. . ¡Entra ya!</t>
         </is>
       </c>
       <c r="N9" s="2" t="n">
@@ -1129,72 +1129,72 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Tubo solar VELUX flexible de 35 cm para tejado inclinado: luz natural en baños, pasillos y estancias sin ventanas. Distribuidor oficial VELUX.</t>
+          <t>Escaleras rectas de madera para interior y altillos: modelos Maydisa resistentes y fáciles de montar. Consulta medidas y precios. Envío a toda España.</t>
         </is>
       </c>
       <c r="P9" s="2" t="n">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>Título cortado («Cubierta I»). «tubo solar velux» en puesto 5 con 0 clics: gran margen.</t>
-        </is>
-      </c>
-      <c r="R9" s="2" t="n"/>
-      <c r="S9" s="2" t="n"/>
+          <t>escalera de madera interior / escalera interior de madera (770/mes): URL objetivo de la estrategia.</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>3 · opcional, desde 10-dic</t>
+          <t>2 · desde 19-nov</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://aluminio-carpinteria.com/ventanas-de-tejado-roto-pivotantes/305-ventanas-de-tejado-roto-r45-pivotante.html</t>
+          <t>https://aluminio-carpinteria.com/580-tubo-solar-velux</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Producto</t>
+          <t>Categoría</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1481</v>
+        <v>762</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>0.1</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>8.5</v>
+        <v>38.2</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>ventanas roto; velux roto</t>
+          <t>tubo solar (1.000/mes) y tubo solar velux (240/mes)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Ventana Tejado Pivotante Roto R45 Madera | Aluminios Olmedo</t>
+          <t>VELUX Tubo Solar | Ilumina Espacios Oscuros | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Ventana de Tejado Roto R45 Pivotante | Aluminios Olmedo</t>
+          <t>Tubo Solar VELUX Rígido y Flexible: Precios | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L10" s="2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Ventana de tejado pivotante Roto R45 en madera lacada. Apertura giratoria en eje central. Distribuidor oficial Roto en Aluminios Olmedo. Envío a España.</t>
+          <t>Instala un velux tubo solar y lleva luz natural a baños y pasillos sin ventanas. Ahorra energía con un tubo solar velux rígido o flexible. ¡Consúltanos!</t>
         </is>
       </c>
       <c r="N10" s="2" t="n">
@@ -1202,19 +1202,19 @@
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>Ventana de tejado Roto R45 pivotante en madera lacada: abre en eje central y se limpia desde dentro. Distribuidor oficial Roto, envío a toda España.</t>
+          <t>Tubo solar VELUX rígido o flexible para tejado inclinado o plano: luz natural en baños y pasillos sin ventanas. Distribuidor oficial VELUX.</t>
         </is>
       </c>
       <c r="P10" s="2" t="n">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>Sale por «ventanas roto» (561 impresiones). Esa búsqueda debe ganarla la categoría 504 (tarea 3.2).</t>
-        </is>
-      </c>
-      <c r="R10" s="2" t="n"/>
-      <c r="S10" s="2" t="n"/>
+          <t>tubo solar (1.000/mes) y tubo solar velux (240/mes): URL objetivo de la estrategia; hoy en posición 38.</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://aluminio-carpinteria.com/persianas-velux/10-velux-persianas-solares-ssl.html</t>
+          <t>https://aluminio-carpinteria.com/tubo-solar-velux-cubierta-inclinada/300-tubo-solar-velux-o-35cm-flexible-cubierta-inclinada.html</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1233,25 +1233,25 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1273</v>
+        <v>1805</v>
       </c>
       <c r="E11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="F11" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>13.5</v>
-      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>persiana solar velux; persianas para velux; persianas para velux baratas</t>
+          <t>tubo solar velux; tubo solar; tubo solar velux precio</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Persiana Solar VELUX SSL para Ventanas de | Aluminios Olmedo</t>
+          <t>Tubo Solar Flexible VELUX 35cm Cubierta I | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
@@ -1259,31 +1259,31 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Persiana Solar VELUX SSL sin Obra | Aluminios Olmedo</t>
+          <t>Tubo Solar VELUX 35 cm Flexible | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L11" s="2" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Persiana exterior solar VELUX SSL para ventanas de tejado. Funciona con energía solar sin obra eléctrica. Distribuidor oficial VELUX.</t>
+          <t>Tubo solar flexible VELUX Ø 35cm para cubierta inclinada. Rodea obstáculos fácilmente. Lleva luz natural al interior. Distribuidor oficial VELUX.</t>
         </is>
       </c>
       <c r="N11" s="2" t="n">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>Persiana solar VELUX SSL para ventanas de tejado: funciona con energía solar, sin cables ni obra eléctrica. Oscurecimiento total. Distribuidor oficial VELUX.</t>
+          <t>Tubo solar VELUX flexible de 35 cm para tejado inclinado: luz natural en baños, pasillos y estancias sin ventanas. Distribuidor oficial VELUX.</t>
         </is>
       </c>
       <c r="P11" s="2" t="n">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>Título cortado («Ventanas de»).</t>
+          <t>Título cortado («Cubierta I»). «tubo solar velux» en puesto 5 con 0 clics: gran margen.</t>
         </is>
       </c>
       <c r="R11" s="2" t="n"/>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://aluminio-carpinteria.com/ventanas-de-tejado-roto-pivotantes/307-ventanas-de-tejado-roto-r48s-pivotante-vidrio-seguridad.html</t>
+          <t>https://aluminio-carpinteria.com/ventanas-de-tejado-roto-pivotantes/305-ventanas-de-tejado-roto-r45-pivotante.html</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1306,61 +1306,207 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1194</v>
+        <v>1481</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>9.800000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>ventanas roto; ventanas de tejado roto; ventanas de tejado roto precios</t>
+          <t>ventanas roto; velux roto</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Ventana Tejado Pivotante Roto R48S Vidrio | Aluminios Olmedo</t>
+          <t>Ventana Tejado Pivotante Roto R45 Madera | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Ventana Roto R48S Vidrio Seguridad | Aluminios Olmedo</t>
+          <t>Roto R45 Pivotante de Madera: Precio y Medidas | Aluminios Olmedo</t>
         </is>
       </c>
       <c r="L12" s="2" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Ventana de tejado pivotante Roto R48S con vidrio laminado de seguridad. Mayor protección frente a rotura. Distribuidor oficial Roto.</t>
+          <t>Ventana de tejado pivotante Roto R45 en madera lacada. Apertura giratoria en eje central. Distribuidor oficial Roto en Aluminios Olmedo. Envío a España.</t>
         </is>
       </c>
       <c r="N12" s="2" t="n">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Ventana de tejado Roto R48S pivotante con vidrio laminado de seguridad, más protección frente a roturas. Consulta precio y medidas. Distribuidor oficial Roto.</t>
+          <t>Ventana de tejado Roto R45 pivotante en madera lacada: abre en eje central y se limpia desde dentro. Distribuidor oficial Roto, envío a toda España.</t>
         </is>
       </c>
       <c r="P12" s="2" t="n">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>Título cortado («Vidrio»).</t>
+          <t>Se evita «ventanas de tejado roto» (es de la 504).</t>
         </is>
       </c>
       <c r="R12" s="2" t="n"/>
       <c r="S12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>3 · opcional, desde 10-dic</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>https://aluminio-carpinteria.com/persianas-velux/10-velux-persianas-solares-ssl.html</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>1273</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>persiana solar velux; persianas para velux; persianas para velux baratas</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Persiana Solar VELUX SSL para Ventanas de | Aluminios Olmedo</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Persiana Solar VELUX SSL sin Obra | Aluminios Olmedo</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Persiana exterior solar VELUX SSL para ventanas de tejado. Funciona con energía solar sin obra eléctrica. Distribuidor oficial VELUX.</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>133</v>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>Persiana solar VELUX SSL para ventanas de tejado: funciona con energía solar, sin cables ni obra eléctrica. Oscurecimiento total. Distribuidor oficial VELUX.</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>Título cortado («Ventanas de»).</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="n"/>
+      <c r="S13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>3 · opcional, desde 10-dic</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>https://aluminio-carpinteria.com/ventanas-de-tejado-roto-pivotantes/307-ventanas-de-tejado-roto-r48s-pivotante-vidrio-seguridad.html</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>1194</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>ventanas roto; ventanas de tejado roto; ventanas de tejado roto precios</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Ventana Tejado Pivotante Roto R48S Vidrio | Aluminios Olmedo</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Roto R48S Pivotante Vidrio de Seguridad: Precio | Aluminios Olmedo</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Ventana de tejado pivotante Roto R48S con vidrio laminado de seguridad. Mayor protección frente a rotura. Distribuidor oficial Roto.</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>Ventana de tejado Roto R48S pivotante con vidrio laminado de seguridad, más protección frente a roturas. Consulta precio y medidas. Distribuidor oficial Roto.</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>158</v>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>Se evita «ventanas de tejado roto» (es de la 504).</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="n"/>
+      <c r="S14" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1373,7 +1519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1503,6 +1649,20 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>https://aluminio-carpinteria.com/560-escaleras-rectas-madera</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>https://aluminio-carpinteria.com/580-tubo-solar-velux</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Títulos: fechas de las tandas relativas al día en que se aplique la tanda 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Le6dThhENh6Yrnr8uFDqix
</commit_message>
<xml_diff>
--- a/entregables/Titulos-metas-2026-10-29.xlsx
+++ b/entregables/Titulos-metas-2026-10-29.xlsx
@@ -562,7 +562,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>1 · ahora</t>
+          <t>1 · próxima sesión</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1 · ahora</t>
+          <t>1 · próxima sesión</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>1 · ahora</t>
+          <t>1 · próxima sesión</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -781,7 +781,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1 · ahora</t>
+          <t>1 · próxima sesión</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>1 · ahora</t>
+          <t>1 · próxima sesión</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2 · desde 19-nov</t>
+          <t>2 · 3 semanas después de la tanda 1</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1000,7 +1000,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2 · desde 19-nov</t>
+          <t>2 · 3 semanas después de la tanda 1</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1073,7 +1073,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2 · desde 19-nov</t>
+          <t>2 · 3 semanas después de la tanda 1</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1146,7 +1146,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2 · desde 19-nov</t>
+          <t>2 · 3 semanas después de la tanda 1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1219,7 +1219,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>3 · opcional, desde 10-dic</t>
+          <t>3 · opcional, 3 semanas después de la tanda 2</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1292,7 +1292,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>3 · opcional, desde 10-dic</t>
+          <t>3 · opcional, 3 semanas después de la tanda 2</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1365,7 +1365,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>3 · opcional, desde 10-dic</t>
+          <t>3 · opcional, 3 semanas después de la tanda 2</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1438,7 +1438,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>3 · opcional, desde 10-dic</t>
+          <t>3 · opcional, 3 semanas después de la tanda 2</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">

</xml_diff>